<commit_message>
sync with new updates
</commit_message>
<xml_diff>
--- a/interview/Coding Summary.xlsx
+++ b/interview/Coding Summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/haoyug1/research/ethics_developer_interview/replication-package/interview/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40B040AA-3001-E24B-8740-B5AF9FBCF696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{338DBD0E-9888-5446-BC0F-779451596D3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3400" yWindow="22360" windowWidth="30240" windowHeight="17660" xr2:uid="{E46B4BFE-8D2E-C342-BCC6-87F284AE669C}"/>
+    <workbookView xWindow="3400" yWindow="22360" windowWidth="30240" windowHeight="17660" activeTab="5" xr2:uid="{E46B4BFE-8D2E-C342-BCC6-87F284AE669C}"/>
   </bookViews>
   <sheets>
     <sheet name="RQ1 Concerns" sheetId="1" r:id="rId1"/>
@@ -2006,9 +2006,6 @@
     <t>Difficuly to communicate safety terminologies between different stakeholders</t>
   </si>
   <si>
-    <t>Human Software Interaction Concerns</t>
-  </si>
-  <si>
     <t>Consideration of malicious use of the software</t>
   </si>
   <si>
@@ -2304,9 +2301,6 @@
   </si>
   <si>
     <t>barriers to technical understanding and information access</t>
-  </si>
-  <si>
-    <t>Insufficient policy and systematic methods issue (safety policy processing gap)</t>
   </si>
   <si>
     <t>Relying on external parties and resources</t>
@@ -2439,6 +2433,12 @@
   </si>
   <si>
     <t>As we are also going to organise codes on the AI software development process, this provides insights on what process contain more problems, or are being most focused on.</t>
+  </si>
+  <si>
+    <t>Misuse and Exploitation Concerns</t>
+  </si>
+  <si>
+    <t>Safety policy interpretation gap</t>
   </si>
 </sst>
 </file>
@@ -3125,7 +3125,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B21" t="s">
         <v>30</v>
@@ -3268,7 +3268,7 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B34" t="s">
         <v>47</v>
@@ -3554,7 +3554,7 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B60" t="s">
         <v>435</v>
@@ -3617,10 +3617,10 @@
   <sheetData>
     <row r="1" spans="1:13" ht="22" x14ac:dyDescent="0.3">
       <c r="B1" s="3" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
@@ -3631,7 +3631,7 @@
         <v>61</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>101</v>
@@ -3646,7 +3646,7 @@
         <v>61</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>100</v>
@@ -3663,7 +3663,7 @@
         <v>62</v>
       </c>
       <c r="C3" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="D3" t="s">
         <v>117</v>
@@ -3675,13 +3675,13 @@
         <v>117</v>
       </c>
       <c r="H3" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="I3" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="J3" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="K3" t="s">
         <v>128</v>
@@ -3701,7 +3701,7 @@
         <v>64</v>
       </c>
       <c r="C4" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="D4" t="s">
         <v>117</v>
@@ -3713,13 +3713,13 @@
         <v>118</v>
       </c>
       <c r="H4" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="I4" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="J4" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="K4" t="s">
         <v>128</v>
@@ -3736,10 +3736,10 @@
         <v>65</v>
       </c>
       <c r="B5" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="C5" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D5" t="s">
         <v>118</v>
@@ -3751,13 +3751,13 @@
         <v>119</v>
       </c>
       <c r="H5" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="I5" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="J5" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="K5" t="s">
         <v>128</v>
@@ -3766,7 +3766,7 @@
         <v>130</v>
       </c>
       <c r="M5" t="s">
-        <v>654</v>
+        <v>791</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
@@ -3777,7 +3777,7 @@
         <v>60</v>
       </c>
       <c r="C6" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="D6" t="s">
         <v>118</v>
@@ -3792,10 +3792,10 @@
         <v>122</v>
       </c>
       <c r="I6" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="J6" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="K6" t="s">
         <v>129</v>
@@ -3809,7 +3809,7 @@
         <v>68</v>
       </c>
       <c r="C7" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="D7" t="s">
         <v>118</v>
@@ -3824,10 +3824,10 @@
         <v>84</v>
       </c>
       <c r="I7" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="J7" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="K7" t="s">
         <v>129</v>
@@ -3841,7 +3841,7 @@
         <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="D8" t="s">
         <v>119</v>
@@ -3856,10 +3856,10 @@
         <v>125</v>
       </c>
       <c r="I8" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="J8" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="K8" t="s">
         <v>129</v>
@@ -3873,7 +3873,7 @@
         <v>236</v>
       </c>
       <c r="C9" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="D9" t="s">
         <v>119</v>
@@ -3885,13 +3885,13 @@
         <v>124</v>
       </c>
       <c r="H9" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="I9" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="J9" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="K9" t="s">
         <v>130</v>
@@ -3905,7 +3905,7 @@
         <v>75</v>
       </c>
       <c r="C10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="D10" t="s">
         <v>118</v>
@@ -3920,10 +3920,10 @@
         <v>127</v>
       </c>
       <c r="I10" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="J10" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="K10" t="s">
         <v>130</v>
@@ -3937,7 +3937,7 @@
         <v>77</v>
       </c>
       <c r="C11" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D11" t="s">
         <v>118</v>
@@ -3954,7 +3954,7 @@
         <v>22</v>
       </c>
       <c r="C12" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="D12" t="s">
         <v>120</v>
@@ -3971,7 +3971,7 @@
         <v>81</v>
       </c>
       <c r="C13" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="D13" t="s">
         <v>120</v>
@@ -3988,7 +3988,7 @@
         <v>82</v>
       </c>
       <c r="C14" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="D14" t="s">
         <v>120</v>
@@ -4005,7 +4005,7 @@
         <v>85</v>
       </c>
       <c r="C15" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="D15" t="s">
         <v>121</v>
@@ -4022,7 +4022,7 @@
         <v>87</v>
       </c>
       <c r="C16" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="D16" t="s">
         <v>121</v>
@@ -4039,7 +4039,7 @@
         <v>89</v>
       </c>
       <c r="C17" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="D17" t="s">
         <v>121</v>
@@ -4056,7 +4056,7 @@
         <v>90</v>
       </c>
       <c r="C18" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="D18" t="s">
         <v>121</v>
@@ -4073,7 +4073,7 @@
         <v>94</v>
       </c>
       <c r="C19" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="D19" t="s">
         <v>121</v>
@@ -4090,7 +4090,7 @@
         <v>49</v>
       </c>
       <c r="C20" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="D20" t="s">
         <v>123</v>
@@ -4107,7 +4107,7 @@
         <v>552</v>
       </c>
       <c r="C21" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="D21" t="s">
         <v>123</v>
@@ -4124,7 +4124,7 @@
         <v>99</v>
       </c>
       <c r="C22" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="D22" t="s">
         <v>123</v>
@@ -4141,7 +4141,7 @@
         <v>103</v>
       </c>
       <c r="C23" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="D23" t="s">
         <v>124</v>
@@ -4158,7 +4158,7 @@
         <v>115</v>
       </c>
       <c r="C24" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="D24" t="s">
         <v>126</v>
@@ -4172,10 +4172,10 @@
         <v>106</v>
       </c>
       <c r="B25" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="C25" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="D25" t="s">
         <v>126</v>
@@ -4192,7 +4192,7 @@
         <v>110</v>
       </c>
       <c r="C26" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="D26" t="s">
         <v>124</v>
@@ -4209,7 +4209,7 @@
         <v>420</v>
       </c>
       <c r="C27" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="D27" t="s">
         <v>124</v>
@@ -4226,7 +4226,7 @@
         <v>114</v>
       </c>
       <c r="C28" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="D28" t="s">
         <v>124</v>
@@ -4243,7 +4243,7 @@
         <v>107</v>
       </c>
       <c r="C29" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="D29" t="s">
         <v>124</v>
@@ -4260,7 +4260,7 @@
         <v>551</v>
       </c>
       <c r="C30" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="D30" t="s">
         <v>126</v>
@@ -4277,7 +4277,7 @@
         <v>555</v>
       </c>
       <c r="C31" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="D31" t="s">
         <v>124</v>
@@ -5380,7 +5380,7 @@
         <v>12</v>
       </c>
       <c r="C98" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.2">
@@ -5407,7 +5407,7 @@
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="B101" t="s">
         <v>8</v>
@@ -6430,7 +6430,7 @@
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B194" t="s">
         <v>454</v>
@@ -6459,10 +6459,10 @@
   <sheetData>
     <row r="1" spans="1:11" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
@@ -6511,7 +6511,7 @@
         <v>351</v>
       </c>
       <c r="G3" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="H3" t="s">
         <v>129</v>
@@ -6520,7 +6520,7 @@
         <v>128</v>
       </c>
       <c r="K3" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
@@ -6540,7 +6540,7 @@
         <v>352</v>
       </c>
       <c r="G4" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="H4" t="s">
         <v>129</v>
@@ -6549,7 +6549,7 @@
         <v>129</v>
       </c>
       <c r="K4" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
@@ -6578,7 +6578,7 @@
         <v>130</v>
       </c>
       <c r="K5" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
@@ -6598,7 +6598,7 @@
         <v>354</v>
       </c>
       <c r="G6" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="H6" t="s">
         <v>128</v>
@@ -6607,7 +6607,7 @@
         <v>373</v>
       </c>
       <c r="K6" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
@@ -6627,7 +6627,7 @@
         <v>355</v>
       </c>
       <c r="G7" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="H7" t="s">
         <v>128</v>
@@ -6636,7 +6636,7 @@
         <v>628</v>
       </c>
       <c r="K7" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
@@ -6653,10 +6653,10 @@
         <v>123</v>
       </c>
       <c r="F8" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="G8" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="H8" t="s">
         <v>628</v>
@@ -6679,7 +6679,7 @@
         <v>356</v>
       </c>
       <c r="G9" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="H9" t="s">
         <v>129</v>
@@ -6702,7 +6702,7 @@
         <v>358</v>
       </c>
       <c r="G10" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="H10" t="s">
         <v>129</v>
@@ -6722,10 +6722,10 @@
         <v>359</v>
       </c>
       <c r="F11" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="G11" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="H11" t="s">
         <v>130</v>
@@ -6748,7 +6748,7 @@
         <v>361</v>
       </c>
       <c r="G12" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="H12" t="s">
         <v>130</v>
@@ -6771,7 +6771,7 @@
         <v>300</v>
       </c>
       <c r="G13" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="H13" t="s">
         <v>628</v>
@@ -6791,10 +6791,10 @@
         <v>363</v>
       </c>
       <c r="F14" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="G14" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="H14" t="s">
         <v>130</v>
@@ -6817,7 +6817,7 @@
         <v>365</v>
       </c>
       <c r="G15" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="H15" t="s">
         <v>373</v>
@@ -6840,7 +6840,7 @@
         <v>370</v>
       </c>
       <c r="G16" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="H16" t="s">
         <v>373</v>
@@ -6863,7 +6863,7 @@
         <v>371</v>
       </c>
       <c r="G17" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="H17" t="s">
         <v>130</v>
@@ -7413,7 +7413,7 @@
         <v>348</v>
       </c>
       <c r="B67" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C67" t="s">
         <v>126</v>
@@ -7611,7 +7611,7 @@
         <v>588</v>
       </c>
       <c r="B85" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="C85" t="s">
         <v>364</v>
@@ -7732,7 +7732,7 @@
         <v>615</v>
       </c>
       <c r="B96" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="C96" t="s">
         <v>118</v>
@@ -7795,10 +7795,10 @@
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
+        <v>662</v>
+      </c>
+      <c r="B102" t="s">
         <v>663</v>
-      </c>
-      <c r="B102" t="s">
-        <v>664</v>
       </c>
       <c r="C102" t="s">
         <v>124</v>
@@ -8393,7 +8393,7 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B53" t="s">
         <v>26</v>
@@ -8404,7 +8404,7 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="B54" t="s">
         <v>435</v>
@@ -8435,10 +8435,10 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
@@ -8493,7 +8493,7 @@
         <v>630</v>
       </c>
       <c r="H3" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="I3" t="s">
         <v>128</v>
@@ -8525,10 +8525,10 @@
         <v>118</v>
       </c>
       <c r="G4" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="H4" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="I4" t="s">
         <v>628</v>
@@ -8563,7 +8563,7 @@
         <v>629</v>
       </c>
       <c r="H5" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="I5" t="s">
         <v>128</v>
@@ -8572,7 +8572,7 @@
         <v>130</v>
       </c>
       <c r="L5" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="M5" t="s">
         <v>423</v>
@@ -8595,10 +8595,10 @@
         <v>120</v>
       </c>
       <c r="G6" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="H6" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="I6" t="s">
         <v>129</v>
@@ -8633,7 +8633,7 @@
         <v>635</v>
       </c>
       <c r="H7" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="I7" t="s">
         <v>129</v>
@@ -8642,7 +8642,7 @@
         <v>628</v>
       </c>
       <c r="L7" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="M7" t="s">
         <v>425</v>
@@ -8665,10 +8665,10 @@
         <v>123</v>
       </c>
       <c r="G8" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="H8" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="I8" t="s">
         <v>129</v>
@@ -8691,10 +8691,10 @@
         <v>124</v>
       </c>
       <c r="G9" t="s">
-        <v>754</v>
+        <v>792</v>
       </c>
       <c r="H9" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="I9" t="s">
         <v>130</v>
@@ -8720,7 +8720,7 @@
         <v>643</v>
       </c>
       <c r="H10" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="I10" t="s">
         <v>130</v>
@@ -8743,10 +8743,10 @@
         <v>359</v>
       </c>
       <c r="G11" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="H11" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="I11" t="s">
         <v>373</v>
@@ -8769,10 +8769,10 @@
         <v>360</v>
       </c>
       <c r="G12" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="H12" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="I12" t="s">
         <v>373</v>
@@ -8798,7 +8798,7 @@
         <v>652</v>
       </c>
       <c r="H13" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="I13" t="s">
         <v>628</v>
@@ -9117,7 +9117,7 @@
         <v>284</v>
       </c>
       <c r="B36" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="C36" t="s">
         <v>118</v>
@@ -9131,7 +9131,7 @@
         <v>286</v>
       </c>
       <c r="B37" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="C37" t="s">
         <v>359</v>
@@ -9156,122 +9156,122 @@
   <sheetData>
     <row r="1" spans="1:2" ht="27" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="27" x14ac:dyDescent="0.35">
       <c r="A2" s="4"/>
       <c r="B2" s="7" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="23" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="7"/>
       <c r="B3" s="7" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="7"/>
       <c r="B4" s="7" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="24" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="24" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="24" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="24" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="24" x14ac:dyDescent="0.3">
       <c r="A10" s="5"/>
       <c r="B10" s="6" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="24" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
       <c r="B11" s="6" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="24" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="6" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="24" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
       <c r="B13" s="6" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="24" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="B14" s="6" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="24" x14ac:dyDescent="0.3">
       <c r="A15" s="6"/>
       <c r="B15" s="6" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6"/>
       <c r="B18" s="6" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="24" x14ac:dyDescent="0.3">
       <c r="A19" s="6"/>
       <c r="B19" s="6" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="24" x14ac:dyDescent="0.3">
       <c r="A20" s="6"/>
       <c r="B20" s="6" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
     </row>
   </sheetData>

</xml_diff>